<commit_message>
update schema by qrest_data
</commit_message>
<xml_diff>
--- a/examples/benchmark_cases/case04_pdf_xlsx/source/monitoring.xlsx
+++ b/examples/benchmark_cases/case04_pdf_xlsx/source/monitoring.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Devices" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Elevation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channels" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,41 +414,147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>InstrumentID</t>
+          <t>Index</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>InstrumentType</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Model</t>
+          <t>Elevation</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>INS-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>DataAcquisitionSystem</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>QDA-2000</t>
-        </is>
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="n">
+        <v>-2.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="n">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="n">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="n">
+        <v>24.3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>27.6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="n">
+        <v>34.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="n">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="n">
+        <v>40.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="n">
+        <v>44.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="n">
+        <v>47.4</v>
       </c>
     </row>
   </sheetData>
@@ -463,186 +568,684 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>SensorID</t>
+          <t>ChannelNo</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>InstrumentID</t>
+          <t>ChannelID</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Floor</t>
+          <t>DeviceType</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>Measurand</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Azimuth</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Z</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>S001</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>INS-001</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>90</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-2.7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>S002</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>INS-001</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>90</v>
+      </c>
+      <c r="G3" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-2.7</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>S003</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>INS-001</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>S05</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Z</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ChannelID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>SensorID</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ChannelNumber</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CH-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>S001</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CH-002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>S002</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CH-003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>S003</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>3</v>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-2.7</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CH-004</t>
-        </is>
+      <c r="A5" t="n">
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>S001</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>4</v>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>90</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>90</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>90</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>90</v>
+      </c>
+      <c r="G12" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>90</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I14" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>90</v>
+      </c>
+      <c r="G15" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>30.9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>90</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>44.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>90</v>
+      </c>
+      <c r="G18" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I18" t="n">
+        <v>44.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Acceleration</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-4.2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>44.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>